<commit_message>
electronic: V4 main board refresh
Updated KiCad project files, board notes and BOM, a combined board image, and
KiCad's backup folder. The stale fp-info-cache is dropped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Electronic/SimInvent_PCBs/Main_Board/SimInvent_FFB_Yoke_Main_Board_V4_BOM.xlsx
+++ b/Electronic/SimInvent_PCBs/Main_Board/SimInvent_FFB_Yoke_Main_Board_V4_BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Superuser\Documents\FlightSim\Force Feedback Yoke\SimInvent FFB Yoke Main Board V4\GERBERS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Superuser\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{964308C6-424D-4846-ADA8-BF416342E6E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6458F60-4820-406F-AAB1-3AC5FAE012E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18290" yWindow="1600" windowWidth="21400" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2620" yWindow="2620" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SimInvent_FFB_Yoke_Main_Boar_BO" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="84">
   <si>
     <t>'Qty'</t>
   </si>
@@ -225,9 +225,6 @@
     <t>C130026</t>
   </si>
   <si>
-    <t>C482347</t>
-  </si>
-  <si>
     <t xml:space="preserve">Buzzer_Beeper:Buzzer6mm      </t>
   </si>
   <si>
@@ -235,15 +232,6 @@
   </si>
   <si>
     <t>D2</t>
-  </si>
-  <si>
-    <t>1N4001</t>
-  </si>
-  <si>
-    <t>SMA DO-214AC</t>
-  </si>
-  <si>
-    <t>C727079</t>
   </si>
   <si>
     <t>DS1023-2*12SF11</t>
@@ -281,6 +269,15 @@
   </si>
   <si>
     <t>C19702</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> DO NOT POPULATE</t>
+  </si>
+  <si>
+    <t>C96256</t>
   </si>
 </sst>
 </file>
@@ -1159,13 +1156,13 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1182,7 +1179,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -1199,7 +1196,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -1360,7 +1357,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
         <v>35</v>
@@ -1411,7 +1408,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>50</v>
@@ -1428,7 +1425,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B18" t="s">
         <v>62</v>
@@ -1479,16 +1476,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
-      </c>
-      <c r="D21" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -1496,13 +1490,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C22" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>57</v>
@@ -1513,16 +1507,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D23" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E23">
         <v>1</v>

</xml_diff>